<commit_message>
chore: backup pre clean install
</commit_message>
<xml_diff>
--- a/docs/MTB Montada R$5.000.xlsx
+++ b/docs/MTB Montada R$5.000.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\junio\OneDrive\Área de Trabalho\Pedal\MTB R$5.000\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/me/Sites/bicicleta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A474B95-6E1F-41A9-A097-63D36750E961}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B1EF727-6A4C-A642-833B-45F033F88218}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="19420" windowHeight="15580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,17 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -310,8 +321,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
-    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -594,22 +605,22 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:K25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.140625" customWidth="1"/>
+    <col min="1" max="1" width="15.1640625" customWidth="1"/>
     <col min="2" max="2" width="35" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" customWidth="1"/>
-    <col min="5" max="5" width="3.7109375" customWidth="1"/>
-    <col min="6" max="6" width="17.42578125" customWidth="1"/>
-    <col min="7" max="7" width="3.7109375" customWidth="1"/>
-    <col min="8" max="8" width="16.140625" customWidth="1"/>
-    <col min="9" max="9" width="3.7109375" customWidth="1"/>
-    <col min="10" max="10" width="22.140625" customWidth="1"/>
-    <col min="11" max="11" width="3.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21.5" customWidth="1"/>
+    <col min="4" max="4" width="19.5" customWidth="1"/>
+    <col min="5" max="5" width="3.6640625" customWidth="1"/>
+    <col min="6" max="6" width="17.5" customWidth="1"/>
+    <col min="7" max="7" width="3.6640625" customWidth="1"/>
+    <col min="8" max="8" width="16.1640625" customWidth="1"/>
+    <col min="9" max="9" width="3.6640625" customWidth="1"/>
+    <col min="10" max="10" width="22.1640625" customWidth="1"/>
+    <col min="11" max="11" width="3.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
       <c r="B1" s="1" t="s">
         <v>20</v>
@@ -628,7 +639,7 @@
       <c r="J1" s="5"/>
       <c r="K1" s="5"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -649,7 +660,7 @@
       <c r="J2" s="5"/>
       <c r="K2" s="5"/>
     </row>
-    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
@@ -668,7 +679,7 @@
       <c r="J3" s="5"/>
       <c r="K3" s="5"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -689,7 +700,7 @@
       <c r="J4" s="5"/>
       <c r="K4" s="5"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -710,7 +721,7 @@
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
@@ -731,14 +742,14 @@
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="10" t="s">
         <v>41</v>
       </c>
       <c r="D7" s="4">
@@ -753,7 +764,7 @@
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>25</v>
       </c>
@@ -772,7 +783,7 @@
       <c r="J8" s="5"/>
       <c r="K8" s="5"/>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
@@ -791,7 +802,7 @@
       <c r="J9" s="5"/>
       <c r="K9" s="5"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
@@ -810,7 +821,7 @@
       <c r="J10" s="5"/>
       <c r="K10" s="5"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
@@ -829,7 +840,7 @@
       <c r="J11" s="5"/>
       <c r="K11" s="5"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
@@ -851,7 +862,7 @@
       <c r="J12" s="5"/>
       <c r="K12" s="5"/>
     </row>
-    <row r="13" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>19</v>
       </c>
@@ -870,7 +881,7 @@
       <c r="J13" s="5"/>
       <c r="K13" s="5"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -891,7 +902,7 @@
       <c r="J14" s="5"/>
       <c r="K14" s="5"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
@@ -913,7 +924,7 @@
       <c r="J15" s="5"/>
       <c r="K15" s="5"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -934,7 +945,7 @@
       <c r="J16" s="5"/>
       <c r="K16" s="5"/>
     </row>
-    <row r="17" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -955,7 +966,7 @@
       <c r="J17" s="5"/>
       <c r="K17" s="5"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -976,7 +987,7 @@
       <c r="J18" s="5"/>
       <c r="K18" s="5"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>12</v>
       </c>
@@ -997,7 +1008,7 @@
       <c r="J19" s="5"/>
       <c r="K19" s="5"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>13</v>
       </c>
@@ -1016,7 +1027,7 @@
       <c r="J20" s="5"/>
       <c r="K20" s="5"/>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>23</v>
       </c>
@@ -1035,7 +1046,7 @@
       <c r="J21" s="5"/>
       <c r="K21" s="5"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>14</v>
       </c>
@@ -1054,7 +1065,7 @@
       <c r="J22" s="5"/>
       <c r="K22" s="5"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>15</v>
       </c>
@@ -1073,7 +1084,7 @@
       <c r="J23" s="5"/>
       <c r="K23" s="5"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>26</v>
       </c>
@@ -1095,7 +1106,7 @@
       <c r="J24" s="5"/>
       <c r="K24" s="5"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>17</v>
       </c>
@@ -1114,7 +1125,10 @@
       <c r="K25" s="5"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C7" r:id="rId1" xr:uid="{1CB5CB7A-BD7C-4A47-AE40-BA0A27EEBAF2}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>